<commit_message>
Implement event-based result checker with sport-specific delays
Features:
- Soccer & NBA: Check after 1h 20min
- MLB, NFL, NHL: Check after 3h
- Per-sport timers instead of fixed polling interval
- Automatic result validation and Excel updates
- Telegram alerts for wins/losses/pushes
- Efficient API usage (1 call per pick when result becomes available)
</commit_message>
<xml_diff>
--- a/picks.xlsx
+++ b/picks.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="26">
   <si>
     <t>Date</t>
   </si>
@@ -45,28 +45,16 @@
     <t>Balance</t>
   </si>
   <si>
-    <t>8 Feb</t>
-  </si>
-  <si>
-    <t>SOCCER</t>
-  </si>
-  <si>
-    <t>Club Leon vs. Necaxa</t>
-  </si>
-  <si>
-    <t>Ambos equipos marcan</t>
+    <t>Tipster</t>
+  </si>
+  <si>
+    <t>PICKS TRACKER - SUMMARY</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Tipster</t>
-  </si>
-  <si>
     <t>Abuelo</t>
-  </si>
-  <si>
-    <t>PICKS TRACKER - SUMMARY</t>
   </si>
   <si>
     <t>Cristian Rey</t>
@@ -507,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -546,35 +534,6 @@
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2">
-        <v>1.66</v>
-      </c>
-      <c r="F2">
-        <v>2000</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -683,7 +642,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -701,7 +660,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -723,35 +682,6 @@
       </c>
       <c r="I1" s="1" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2">
-        <v>1.66</v>
-      </c>
-      <c r="G2">
-        <v>2000</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -771,29 +701,29 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="D2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -810,7 +740,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -827,7 +757,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -844,7 +774,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -861,53 +791,53 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -923,7 +853,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B1">
         <v>3</v>

</xml_diff>

<commit_message>
Fix result checker: correct API sport keys, CSV backup, parser cleanup
- Fix soccer API: use correct league keys (soccer_efl_champ instead of
  soccer_england_championship), stop early when match is found
- Add CSV backup (picks_backup.csv) as fallback to prevent data loss
- Fix parser: strip pick phrases (Ambos anotan Sí, etc.) before extracting
  team names so noise words don't leak into match column
- Fix Excel: never delete existing file, normalize date/match comparison
  for result updates, patch ExcelJS data-validations bug
- Add --dry-run and --days2/--days3 flags to test script
- Log API credits remaining on each paid call

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/picks.xlsx
+++ b/picks.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="28">
   <si>
     <t>Date</t>
   </si>
@@ -45,18 +45,30 @@
     <t>Balance</t>
   </si>
   <si>
+    <t>02 Mar</t>
+  </si>
+  <si>
+    <t>SOCCER</t>
+  </si>
+  <si>
+    <t>Sí Birmingham vs. FC Middlesbrough</t>
+  </si>
+  <si>
+    <t>Ambos equipos marcan</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>Tipster</t>
   </si>
   <si>
+    <t>Abuelo</t>
+  </si>
+  <si>
     <t>PICKS TRACKER - SUMMARY</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Abuelo</t>
-  </si>
-  <si>
     <t>Cristian Rey</t>
   </si>
   <si>
@@ -81,13 +93,7 @@
     <t>Win Rate %</t>
   </si>
   <si>
-    <t>0%</t>
-  </si>
-  <si>
     <t>Total Profit/Loss</t>
-  </si>
-  <si>
-    <t>$0.00</t>
   </si>
   <si>
     <t>Yield %</t>
@@ -100,6 +106,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -146,16 +156,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -495,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -536,7 +556,69 @@
         <v>8</v>
       </c>
     </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>1.71</v>
+      </c>
+      <c r="F2">
+        <v>2000</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="2">
+        <f>IF(G2="W",(F2-1)*2000,IF(G2="L",-2000,0))</f>
+      </c>
+      <c r="I2" s="2">
+        <f>H2</f>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3">
+        <v>1.71</v>
+      </c>
+      <c r="F3">
+        <v>2000</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="2">
+        <f>IF(G3="W",(F3-1)*2000,IF(G3="L",-2000,0))</f>
+      </c>
+      <c r="I3" s="2">
+        <f>I2+H3</f>
+      </c>
+    </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="Object]"/>
+    <dataValidation sqref="[object"/>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -642,7 +724,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -660,7 +742,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -684,7 +766,69 @@
         <v>7</v>
       </c>
     </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2">
+        <v>1.71</v>
+      </c>
+      <c r="G2">
+        <v>2000</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="2">
+        <f>IF(H2="W",(G2-1)*2000,IF(H2="L",-2000,0))</f>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3">
+        <v>1.71</v>
+      </c>
+      <c r="G3">
+        <v>2000</v>
+      </c>
+      <c r="H3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="2">
+        <f>IF(H3="W",(G3-1)*2000,IF(H3="L",-2000,0))</f>
+      </c>
+    </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="Object]"/>
+    <dataValidation sqref="[object"/>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -700,144 +844,144 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>10</v>
+      <c r="A1" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>15</v>
       </c>
+      <c r="C2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
+      <c r="A3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="6">
+        <f>COUNTA(Abuelo!A2:A1000)-COUNTA(Abuelo!G2:G1000)</f>
+      </c>
+      <c r="C3" s="6">
+        <f>COUNTA('Cristian Rey'!A2:A1000)-COUNTA('Cristian Rey'!G2:G1000)</f>
+      </c>
+      <c r="D3" s="6">
+        <f>COUNTA('Roberto Rey'!A2:A1000)-COUNTA('Roberto Rey'!G2:G1000)</f>
+      </c>
+      <c r="E3" s="6">
+        <f>B3+C3+D3</f>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
+      <c r="A4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="6">
+        <f>COUNTIF(Abuelo!G:G,"W")</f>
+      </c>
+      <c r="C4" s="6">
+        <f>COUNTIF('Cristian Rey'!G:G,"W")</f>
+      </c>
+      <c r="D4" s="6">
+        <f>COUNTIF('Roberto Rey'!G:G,"W")</f>
+      </c>
+      <c r="E4" s="6">
+        <f>B4+C4+D4</f>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
+      <c r="A5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="6">
+        <f>COUNTIF(Abuelo!G:G,"L")</f>
+      </c>
+      <c r="C5" s="6">
+        <f>COUNTIF('Cristian Rey'!G:G,"L")</f>
+      </c>
+      <c r="D5" s="6">
+        <f>COUNTIF('Roberto Rey'!G:G,"L")</f>
+      </c>
+      <c r="E5" s="6">
+        <f>B5+C5+D5</f>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
+      <c r="A6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="6">
+        <f>COUNTIF(Abuelo!G:G,"P")</f>
+      </c>
+      <c r="C6" s="6">
+        <f>COUNTIF('Cristian Rey'!G:G,"P")</f>
+      </c>
+      <c r="D6" s="6">
+        <f>COUNTIF('Roberto Rey'!G:G,"P")</f>
+      </c>
+      <c r="E6" s="6">
+        <f>B6+C6+D6</f>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" t="s">
-        <v>21</v>
+      <c r="A7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="7">
+        <f>IF((B4+B5)=0,0,B4/(B4+B5))</f>
+      </c>
+      <c r="C7" s="7">
+        <f>IF((C4+C5)=0,0,C4/(C4+C5))</f>
+      </c>
+      <c r="D7" s="7">
+        <f>IF((D4+D5)=0,0,D4/(D4+D5))</f>
+      </c>
+      <c r="E7" s="7">
+        <f>IF((B4+B5+C4+C5+D4+D5)=0,0,(B4+C4+D4)/(B4+B5+C4+C5+D4+D5))</f>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" t="s">
-        <v>23</v>
+      <c r="A8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="8">
+        <f>SUMIF(Abuelo!G:G,"W",Abuelo!H:H)+SUMIF(Abuelo!G:G,"L",Abuelo!H:H)</f>
+      </c>
+      <c r="C8" s="8">
+        <f>SUMIF('Cristian Rey'!G:G,"W",'Cristian Rey'!H:H)+SUMIF('Cristian Rey'!G:G,"L",'Cristian Rey'!H:H)</f>
+      </c>
+      <c r="D8" s="8">
+        <f>SUMIF('Roberto Rey'!G:G,"W",'Roberto Rey'!H:H)+SUMIF('Roberto Rey'!G:G,"L",'Roberto Rey'!H:H)</f>
+      </c>
+      <c r="E8" s="8">
+        <f>B8+C8+D8</f>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" t="s">
-        <v>21</v>
+      <c r="A9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="7">
+        <f>IF(B3=0,0,B8/(B3*2000))</f>
+      </c>
+      <c r="C9" s="7">
+        <f>IF(C3=0,0,C8/(C3*2000))</f>
+      </c>
+      <c r="D9" s="7">
+        <f>IF(D3=0,0,D8/(D3*2000))</f>
+      </c>
+      <c r="E9" s="7">
+        <f>IF(E3=0,0,E8/(E3*2000))</f>
       </c>
     </row>
   </sheetData>
@@ -853,7 +997,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B1">
         <v>3</v>

</xml_diff>